<commit_message>
Versión para Marzo-Mayo 2025
</commit_message>
<xml_diff>
--- a/AA - Calendario de Turnos(version Abril Julio 2026-caculado el 2026-03-05).xlsx
+++ b/AA - Calendario de Turnos(version Abril Julio 2026-caculado el 2026-03-05).xlsx
@@ -2301,7 +2301,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Cabello</t>
+          <t>Ramos</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Gajardo</t>
+          <t xml:space="preserve">  - Gajardo - Cabello</t>
         </is>
       </c>
     </row>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Gajardo</t>
+          <t xml:space="preserve">  - Gajardo - Cabello</t>
         </is>
       </c>
     </row>
@@ -2398,7 +2398,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Gajardo</t>
+          <t xml:space="preserve">  - Gajardo - Cabello</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Gajardo</t>
+          <t xml:space="preserve">  - Gajardo - Cabello</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Gajardo</t>
+          <t xml:space="preserve">  - Gajardo - Cabello</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Gajardo</t>
+          <t xml:space="preserve">  - Gajardo - Cabello</t>
         </is>
       </c>
     </row>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Gajardo</t>
+          <t xml:space="preserve">  - Gajardo - Cabello</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Ramos</t>
+          <t>Salazar</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Gajardo</t>
+          <t xml:space="preserve">  - Gajardo - Cabello</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Gajardo</t>
+          <t xml:space="preserve">  - Gajardo - Cabello</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Salazar</t>
+          <t>Winter</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Winter</t>
+          <t>Abarca</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Abarca</t>
+          <t>Gajardo</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3736,7 +3736,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Gajardo</t>
+          <t>Cabello</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Cabello</t>
+          <t>Ramos</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Ramos</t>
+          <t>Salazar</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -4597,7 +4597,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Salazar</t>
+          <t>Winter</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Winter</t>
+          <t>Abarca</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Abarca</t>
+          <t>Gajardo</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Gajardo</t>
+          <t>Cabello</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">

</xml_diff>